<commit_message>
4.31: marksheets go trainer -> Assessment Officer -> HOD; Excel heading and footer as cells, filled with names, initials and dates; AVG only with all three marks (else C.R.N.M)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/marksheet.xlsx
+++ b/templates/marksheet.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,23 @@
       <b val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="FF0070C0"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe Script"/>
+      <i val="1"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -139,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
@@ -170,6 +187,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFont="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyFont="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyFont="1" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyFont="1" applyBorder="1" applyAlignment="1" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -247,53 +279,32 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <oneCellAnchor>
     <from>
-      <col>0</col>
-      <colOff>0</colOff>
+      <col>3</col>
+      <colOff>885825</colOff>
       <row>0</row>
-      <rowOff>0</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="10458450" cy="1600200"/>
+    <ext cx="952500" cy="952500"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
+        <cNvPr id="1" name="RVNP crest" descr="RVNP crest"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip r:embed="rId1" cstate="print"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="8248650" cy="1133475"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
       </spPr>
     </pic>
     <clientData/>
@@ -590,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A10:L16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.33" customWidth="1" min="1" max="1"/>
@@ -613,9 +624,60 @@
     <row r="4" ht="15.75" customHeight="1"/>
     <row r="5" ht="15.75" customHeight="1"/>
     <row r="6" ht="15.75" customHeight="1"/>
-    <row r="7" ht="15.75" customHeight="1"/>
-    <row r="8" ht="15.75" customHeight="1"/>
-    <row r="9" ht="15.75" customHeight="1"/>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>THE RIFT VALLEY NATIONAL POLYTECHNIC</t>
+        </is>
+      </c>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>DEPARTMENT OF COMPUTING AND INFORMATICS</t>
+        </is>
+      </c>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>CONTINUOUS ASSESSMENT MARKS SHEET PER UNIT OF COMPETENCY</t>
+        </is>
+      </c>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+    </row>
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -770,31 +832,11 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1"/>
-    <row r="18" ht="15.75" customHeight="1"/>
-    <row r="19" ht="15.75" customHeight="1"/>
-    <row r="20" ht="15.75" customHeight="1"/>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="19">
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A9:L9"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="G11:L11"/>
     <mergeCell ref="E14:H14"/>

</xml_diff>